<commit_message>
Added new RDF data schemes and visual schemes for environment-table13-14, and fixed XLSX spreadsheets for environment-table13-14
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table13.xlsx
+++ b/sources/table_normalization/xlsx/environment-table13.xlsx
@@ -912,8 +912,6 @@
     <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="15" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -967,17 +965,15 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="11" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="2" fontId="11" fillId="2" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="11" fillId="2" borderId="3" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="11" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="11" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -987,6 +983,10 @@
     <xf numFmtId="2" fontId="11" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -1294,7 +1294,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2697,152 +2697,152 @@
       <c r="A4" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="56"/>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
-      <c r="I4" s="56"/>
-      <c r="J4" s="56"/>
-      <c r="K4" s="56"/>
-      <c r="L4" s="57"/>
-      <c r="M4" s="58"/>
-      <c r="N4" s="58"/>
-      <c r="O4" s="58"/>
-      <c r="P4" s="56"/>
-      <c r="Q4" s="56"/>
-      <c r="R4" s="56"/>
-      <c r="S4" s="56"/>
-      <c r="T4" s="56"/>
-      <c r="U4" s="56"/>
-      <c r="V4" s="56"/>
-      <c r="W4" s="56"/>
-      <c r="X4" s="56"/>
-      <c r="Y4" s="56"/>
-      <c r="Z4" s="56"/>
-      <c r="AA4" s="56"/>
-      <c r="AB4" s="59"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
+      <c r="E4" s="53"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54"/>
+      <c r="K4" s="54"/>
+      <c r="L4" s="55"/>
+      <c r="M4" s="56"/>
+      <c r="N4" s="56"/>
+      <c r="O4" s="56"/>
+      <c r="P4" s="54"/>
+      <c r="Q4" s="54"/>
+      <c r="R4" s="54"/>
+      <c r="S4" s="54"/>
+      <c r="T4" s="54"/>
+      <c r="U4" s="54"/>
+      <c r="V4" s="54"/>
+      <c r="W4" s="54"/>
+      <c r="X4" s="54"/>
+      <c r="Y4" s="54"/>
+      <c r="Z4" s="54"/>
+      <c r="AA4" s="54"/>
+      <c r="AB4" s="57"/>
     </row>
     <row r="5" spans="1:28" s="4" customFormat="1" ht="29.25" customHeight="1">
-      <c r="A5" s="41"/>
-      <c r="B5" s="63" t="s">
+      <c r="A5" s="69"/>
+      <c r="B5" s="62" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="63"/>
-      <c r="D5" s="64"/>
-      <c r="E5" s="65" t="s">
+      <c r="C5" s="62"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="63"/>
-      <c r="G5" s="64"/>
-      <c r="H5" s="65" t="s">
+      <c r="F5" s="62"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="I5" s="63"/>
-      <c r="J5" s="64"/>
-      <c r="K5" s="65" t="s">
+      <c r="I5" s="62"/>
+      <c r="J5" s="63"/>
+      <c r="K5" s="61" t="s">
         <v>7</v>
       </c>
-      <c r="L5" s="63"/>
-      <c r="M5" s="64"/>
-      <c r="N5" s="65" t="s">
+      <c r="L5" s="62"/>
+      <c r="M5" s="63"/>
+      <c r="N5" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="O5" s="63"/>
-      <c r="P5" s="64"/>
-      <c r="Q5" s="65" t="s">
+      <c r="O5" s="62"/>
+      <c r="P5" s="63"/>
+      <c r="Q5" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="R5" s="63"/>
-      <c r="S5" s="64"/>
-      <c r="T5" s="65" t="s">
+      <c r="R5" s="62"/>
+      <c r="S5" s="63"/>
+      <c r="T5" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="U5" s="63"/>
-      <c r="V5" s="64"/>
-      <c r="W5" s="65" t="s">
+      <c r="U5" s="62"/>
+      <c r="V5" s="63"/>
+      <c r="W5" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="X5" s="63"/>
-      <c r="Y5" s="64"/>
-      <c r="Z5" s="68" t="s">
+      <c r="X5" s="62"/>
+      <c r="Y5" s="63"/>
+      <c r="Z5" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="AA5" s="69"/>
-      <c r="AB5" s="70"/>
+      <c r="AA5" s="65"/>
+      <c r="AB5" s="66"/>
     </row>
     <row r="6" spans="1:28" s="5" customFormat="1">
-      <c r="A6" s="42"/>
-      <c r="B6" s="60" t="s">
+      <c r="A6" s="70"/>
+      <c r="B6" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="66" t="s">
+      <c r="C6" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="67"/>
-      <c r="E6" s="60" t="s">
+      <c r="D6" s="68"/>
+      <c r="E6" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="61" t="s">
+      <c r="F6" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="62"/>
-      <c r="H6" s="60" t="s">
+      <c r="G6" s="60"/>
+      <c r="H6" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="I6" s="61" t="s">
+      <c r="I6" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="62"/>
-      <c r="K6" s="60" t="s">
+      <c r="J6" s="60"/>
+      <c r="K6" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="L6" s="61" t="s">
+      <c r="L6" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="M6" s="62"/>
-      <c r="N6" s="60" t="s">
+      <c r="M6" s="60"/>
+      <c r="N6" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="O6" s="61" t="s">
+      <c r="O6" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="P6" s="62"/>
-      <c r="Q6" s="60" t="s">
+      <c r="P6" s="60"/>
+      <c r="Q6" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="R6" s="61" t="s">
+      <c r="R6" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="S6" s="62"/>
-      <c r="T6" s="60" t="s">
+      <c r="S6" s="60"/>
+      <c r="T6" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="U6" s="61" t="s">
+      <c r="U6" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="V6" s="62"/>
-      <c r="W6" s="60" t="s">
+      <c r="V6" s="60"/>
+      <c r="W6" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="X6" s="61" t="s">
+      <c r="X6" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="Y6" s="62"/>
-      <c r="Z6" s="60" t="s">
+      <c r="Y6" s="60"/>
+      <c r="Z6" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="AA6" s="61" t="s">
+      <c r="AA6" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="AB6" s="62"/>
+      <c r="AB6" s="60"/>
     </row>
     <row r="7" spans="1:28" s="8" customFormat="1">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="41" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="6">
@@ -2851,7 +2851,7 @@
       <c r="C7" s="7">
         <v>2008</v>
       </c>
-      <c r="D7" s="53" t="s">
+      <c r="D7" s="51" t="s">
         <v>15</v>
       </c>
       <c r="E7" s="6">
@@ -2860,7 +2860,7 @@
       <c r="F7" s="7">
         <v>2008</v>
       </c>
-      <c r="G7" s="53" t="s">
+      <c r="G7" s="51" t="s">
         <v>15</v>
       </c>
       <c r="H7" s="6">
@@ -2869,7 +2869,7 @@
       <c r="I7" s="7">
         <v>2008</v>
       </c>
-      <c r="J7" s="53" t="s">
+      <c r="J7" s="51" t="s">
         <v>15</v>
       </c>
       <c r="K7" s="6">
@@ -2878,7 +2878,7 @@
       <c r="L7" s="7">
         <v>2008</v>
       </c>
-      <c r="M7" s="53" t="s">
+      <c r="M7" s="51" t="s">
         <v>15</v>
       </c>
       <c r="N7" s="6">
@@ -2887,7 +2887,7 @@
       <c r="O7" s="7">
         <v>2008</v>
       </c>
-      <c r="P7" s="53" t="s">
+      <c r="P7" s="51" t="s">
         <v>15</v>
       </c>
       <c r="Q7" s="6">
@@ -2896,7 +2896,7 @@
       <c r="R7" s="7">
         <v>2008</v>
       </c>
-      <c r="S7" s="53" t="s">
+      <c r="S7" s="51" t="s">
         <v>15</v>
       </c>
       <c r="T7" s="6">
@@ -2905,7 +2905,7 @@
       <c r="U7" s="7">
         <v>2008</v>
       </c>
-      <c r="V7" s="53" t="s">
+      <c r="V7" s="51" t="s">
         <v>15</v>
       </c>
       <c r="W7" s="6">
@@ -2914,7 +2914,7 @@
       <c r="X7" s="7">
         <v>2008</v>
       </c>
-      <c r="Y7" s="53" t="s">
+      <c r="Y7" s="51" t="s">
         <v>15</v>
       </c>
       <c r="Z7" s="6">
@@ -2923,7 +2923,7 @@
       <c r="AA7" s="7">
         <v>2008</v>
       </c>
-      <c r="AB7" s="53" t="s">
+      <c r="AB7" s="51" t="s">
         <v>15</v>
       </c>
     </row>
@@ -11940,7 +11940,7 @@
       </c>
     </row>
     <row r="118" spans="1:28" s="2" customFormat="1">
-      <c r="A118" s="44" t="s">
+      <c r="A118" s="42" t="s">
         <v>120</v>
       </c>
       <c r="B118" s="29"/>
@@ -11972,7 +11972,7 @@
       <c r="AB118"/>
     </row>
     <row r="119" spans="1:28" s="2" customFormat="1">
-      <c r="A119" s="45" t="s">
+      <c r="A119" s="43" t="s">
         <v>121</v>
       </c>
       <c r="B119" s="31"/>
@@ -12004,7 +12004,7 @@
       <c r="AB119"/>
     </row>
     <row r="120" spans="1:28" s="2" customFormat="1">
-      <c r="A120" s="46" t="s">
+      <c r="A120" s="44" t="s">
         <v>122</v>
       </c>
       <c r="B120" s="32"/>
@@ -12036,7 +12036,7 @@
       <c r="AB120"/>
     </row>
     <row r="121" spans="1:28" s="2" customFormat="1">
-      <c r="A121" s="47" t="s">
+      <c r="A121" s="45" t="s">
         <v>123</v>
       </c>
       <c r="B121" s="34"/>
@@ -12068,7 +12068,7 @@
       <c r="AB121"/>
     </row>
     <row r="122" spans="1:28" s="2" customFormat="1">
-      <c r="A122" s="47" t="s">
+      <c r="A122" s="45" t="s">
         <v>124</v>
       </c>
       <c r="B122" s="34"/>
@@ -12100,7 +12100,7 @@
       <c r="AB122"/>
     </row>
     <row r="123" spans="1:28" s="2" customFormat="1">
-      <c r="A123" s="48" t="s">
+      <c r="A123" s="46" t="s">
         <v>125</v>
       </c>
       <c r="B123" s="34"/>
@@ -12135,12 +12135,12 @@
       <c r="A124" s="31"/>
     </row>
     <row r="125" spans="1:28">
-      <c r="A125" s="45" t="s">
+      <c r="A125" s="43" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="126" spans="1:28">
-      <c r="A126" s="45" t="s">
+      <c r="A126" s="43" t="s">
         <v>127</v>
       </c>
     </row>
@@ -12148,7 +12148,7 @@
       <c r="A127" s="31"/>
     </row>
     <row r="128" spans="1:28">
-      <c r="A128" s="49" t="s">
+      <c r="A128" s="47" t="s">
         <v>128</v>
       </c>
       <c r="B128" s="35"/>
@@ -12168,7 +12168,7 @@
       <c r="U128" s="1"/>
     </row>
     <row r="129" spans="1:21">
-      <c r="A129" s="50" t="s">
+      <c r="A129" s="48" t="s">
         <v>129</v>
       </c>
       <c r="B129" s="35"/>
@@ -12188,7 +12188,7 @@
       <c r="U129" s="1"/>
     </row>
     <row r="130" spans="1:21">
-      <c r="A130" s="50" t="s">
+      <c r="A130" s="48" t="s">
         <v>130</v>
       </c>
       <c r="B130" s="35"/>
@@ -12208,7 +12208,7 @@
       <c r="U130" s="1"/>
     </row>
     <row r="131" spans="1:21">
-      <c r="A131" s="50" t="s">
+      <c r="A131" s="48" t="s">
         <v>131</v>
       </c>
       <c r="B131" s="35"/>
@@ -12228,7 +12228,7 @@
       <c r="U131" s="1"/>
     </row>
     <row r="132" spans="1:21">
-      <c r="A132" s="50" t="s">
+      <c r="A132" s="48" t="s">
         <v>132</v>
       </c>
       <c r="B132" s="35"/>
@@ -12248,7 +12248,7 @@
       <c r="U132" s="1"/>
     </row>
     <row r="133" spans="1:21">
-      <c r="A133" s="51" t="s">
+      <c r="A133" s="49" t="s">
         <v>133</v>
       </c>
       <c r="B133" s="35"/>
@@ -12286,7 +12286,7 @@
       <c r="U134" s="1"/>
     </row>
     <row r="135" spans="1:21">
-      <c r="A135" s="52" t="s">
+      <c r="A135" s="50" t="s">
         <v>134</v>
       </c>
       <c r="B135" s="1"/>
@@ -12316,11 +12316,6 @@
   </sheetData>
   <autoFilter ref="A7:A117"/>
   <mergeCells count="18">
-    <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="Z6:AB6"/>
-    <mergeCell ref="T5:V5"/>
-    <mergeCell ref="W5:Y5"/>
-    <mergeCell ref="Z5:AB5"/>
     <mergeCell ref="Q6:S6"/>
     <mergeCell ref="T6:V6"/>
     <mergeCell ref="B5:D5"/>
@@ -12334,6 +12329,11 @@
     <mergeCell ref="H6:J6"/>
     <mergeCell ref="K6:M6"/>
     <mergeCell ref="N6:P6"/>
+    <mergeCell ref="W6:Y6"/>
+    <mergeCell ref="Z6:AB6"/>
+    <mergeCell ref="T5:V5"/>
+    <mergeCell ref="W5:Y5"/>
+    <mergeCell ref="Z5:AB5"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>

</xml_diff>